<commit_message>
final editing of excel sheet i think
</commit_message>
<xml_diff>
--- a/Proj1_control_signals.xlsx
+++ b/Proj1_control_signals.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="91">
   <si>
     <t xml:space="preserve">Instruction</t>
   </si>
@@ -242,6 +242,57 @@
   </si>
   <si>
     <t xml:space="preserve">XX?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bltu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bgeu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XXXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jalr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lbu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lhu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">srli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">srai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auipc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wfi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">????</t>
   </si>
 </sst>
 </file>
@@ -276,12 +327,18 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -318,7 +375,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -343,6 +400,22 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -360,7 +433,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr defaultColWidth="10.86328125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.88"/>
@@ -1515,7 +1588,759 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P23" s="1"/>
+      <c r="A23" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>1100011</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>1100011</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>101</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>1100011</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>1100011</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>111</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>1101111</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q27" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>1100111</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q28" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q29" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q30" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q31" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>101</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q32" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>110011</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>111</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P33" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q33" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>10011</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>101</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>101</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P34" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q34" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>10011</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>101</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P35" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q35" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>10111</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q36" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C37" s="8"/>
+      <c r="D37" s="9"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>